<commit_message>
19-july before webwright commitment
</commit_message>
<xml_diff>
--- a/features/HCM/CoreHR/WorkForceModelTestData.xlsx
+++ b/features/HCM/CoreHR/WorkForceModelTestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\girdh\Downloads\Playwright_Framwork-20260628T075205Z-3-001\Playwright_Framwork\tests\projectWorkSpaceERP\HCM\CoreHR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10854578\Playwright_Framework\features\HCM\CoreHR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE2C3F4-3070-4429-8A98-6880D749A3BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C70F0B39-1469-4278-B8C7-2CCC79A540C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -130,12 +130,6 @@
     <t>TRUE</t>
   </si>
   <si>
-    <t>Trainee User Functional</t>
-  </si>
-  <si>
-    <t>@+34Ll8I_|ib</t>
-  </si>
-  <si>
     <t>True</t>
   </si>
   <si>
@@ -167,6 +161,12 @@
   </si>
   <si>
     <t>Saudi Arabia</t>
+  </si>
+  <si>
+    <t>HCM_IMPL</t>
+  </si>
+  <si>
+    <t>f%6^9qKN</t>
   </si>
 </sst>
 </file>
@@ -565,30 +565,30 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" style="10" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="13.5546875" style="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="13.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.5546875" style="13" bestFit="1" customWidth="1"/>
-    <col min="22" max="31" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="13.5546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="15.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.54296875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.08984375" style="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="13.54296875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.08984375" style="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="13.54296875" style="14" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.54296875" style="14" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.54296875" style="13" bestFit="1" customWidth="1"/>
+    <col min="22" max="31" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="13.54296875" style="14" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="15.54296875" style="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -692,7 +692,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -700,46 +700,46 @@
         <v>35</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="E2" s="5">
         <v>380871860776</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G2" s="6">
         <v>46023</v>
       </c>
       <c r="H2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" t="s">
         <v>39</v>
-      </c>
-      <c r="I2" t="s">
-        <v>40</v>
-      </c>
-      <c r="J2" t="s">
-        <v>39</v>
-      </c>
-      <c r="K2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="N2" t="s">
-        <v>41</v>
       </c>
       <c r="O2" s="6">
         <v>30683</v>
       </c>
       <c r="P2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Q2" s="5">
         <v>212</v>
@@ -748,29 +748,29 @@
         <v>7123813</v>
       </c>
       <c r="S2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T2" s="5">
         <v>123</v>
       </c>
       <c r="U2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AE2" s="8" t="s">
         <v>44</v>
-      </c>
-      <c r="X2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AE2" s="8" t="s">
-        <v>46</v>
       </c>
       <c r="AF2" s="5"/>
       <c r="AG2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="AH2" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C3" s="4"/>
       <c r="E3" s="9"/>
       <c r="G3" s="3"/>
@@ -785,7 +785,7 @@
       <c r="AF3" s="5"/>
       <c r="AH3" s="5"/>
     </row>
-    <row r="4" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C4" s="4"/>
       <c r="D4" s="1"/>
       <c r="E4" s="9"/>
@@ -800,7 +800,7 @@
       <c r="AF4" s="5"/>
       <c r="AH4" s="5"/>
     </row>
-    <row r="5" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7"/>
       <c r="C5" s="4"/>
       <c r="E5" s="9"/>
@@ -815,7 +815,7 @@
       <c r="AF5" s="5"/>
       <c r="AH5" s="5"/>
     </row>
-    <row r="6" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C6" s="4"/>
       <c r="E6" s="9"/>
       <c r="G6" s="3"/>
@@ -830,7 +830,7 @@
       <c r="AF6" s="5"/>
       <c r="AH6" s="5"/>
     </row>
-    <row r="7" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C7" s="4"/>
       <c r="E7" s="9"/>
       <c r="G7" s="3"/>
@@ -844,7 +844,7 @@
       <c r="AF7" s="5"/>
       <c r="AH7" s="5"/>
     </row>
-    <row r="8" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:34" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C8" s="4"/>
       <c r="E8" s="9"/>
       <c r="G8" s="3"/>

</xml_diff>